<commit_message>
Rate limits, campthca, javascript,ajax, structure drift, session consistency, login wall, honeypot, large batch, monotoring
</commit_message>
<xml_diff>
--- a/public/nexus-product-import-template.xlsx
+++ b/public/nexus-product-import-template.xlsx
@@ -17,6 +17,15 @@
   </si>
   <si>
     <t>EAN</t>
+  </si>
+  <si>
+    <t>SKU</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Your Price</t>
   </si>
   <si>
     <t>Example product (delete this row)</t>
@@ -80,6 +89,9 @@
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -89,13 +101,22 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>